<commit_message>
Fix canonical profile links
</commit_message>
<xml_diff>
--- a/sources/Evidence_Ledger.xlsx
+++ b/sources/Evidence_Ledger.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R306502d942124ad3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flagship Evidence" sheetId="2" r:id="R7289de613d6a4b6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical Repositories" sheetId="3" r:id="Rb8af631f91d34e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ecosystem Summary" sheetId="4" r:id="R55325958bb55429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Professional Record" sheetId="5" r:id="R48a6c868567648d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="6" r:id="Rac04ddf888ee4040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ministry Evidence" sheetId="7" r:id="R3c3bd47ecd3f44ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="8" r:id="Rfcb7f0ccbde2464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="9" r:id="Rbb6a87b3b7284944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="10" r:id="Reee7532f083c4c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2974a50b92bc4972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flagship Evidence" sheetId="2" r:id="Ra09edc9c64594f74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Canonical Repositories" sheetId="3" r:id="R30d5ce290ecc4b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ecosystem Summary" sheetId="4" r:id="R28fe26a40ce94193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Professional Record" sheetId="5" r:id="Rbfa04cbe5fbc4540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="6" r:id="Rbe0b540d1cb946ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ministry Evidence" sheetId="7" r:id="R915c1f52064d464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="8" r:id="R00705ebe5a324417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="9" r:id="Reaa2187e9be54a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="10" r:id="R96ec93c28a4141a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2026,9 +2026,6 @@
     <x:t xml:space="preserve">Subject-supplied / programme context public</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Professional Dossier; https://www.intracen.org/our-work/projects/eu-eac-market-access-upgrade-programme-markup</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Use outcome-level language only.</x:t>
   </x:si>
   <x:si>
@@ -2780,9 +2777,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Public programme context; not employment</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://www.intracen.org/our-work/projects/eu-eac-market-access-upgrade-programme-markup</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Use accurate programme wording.</x:t>
@@ -3924,7 +3918,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2bb6b5f45314831"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc56fa6c8977d4b66"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4634,7 +4628,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>966</x:v>
+        <x:v>964</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -4656,16 +4650,16 @@
     </x:row>
     <x:row r="4" ht="30" hidden="0" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>965</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
+        <x:v>966</x:v>
+      </x:c>
+      <x:c r="C4" s="15" t="s">
         <x:v>967</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
+      <x:c r="D4" s="15" t="s">
         <x:v>968</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
-        <x:v>969</x:v>
-      </x:c>
-      <x:c r="D4" s="15" t="s">
-        <x:v>970</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" hidden="0" customHeight="1">
@@ -4673,13 +4667,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B5" s="11" t="s">
+        <x:v>969</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="s">
+        <x:v>970</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="s">
         <x:v>971</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="s">
-        <x:v>972</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="s">
-        <x:v>973</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" hidden="0" customHeight="1">
@@ -4687,13 +4681,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B6" s="11" t="s">
+        <x:v>972</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="s">
+        <x:v>973</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="s">
         <x:v>974</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="s">
-        <x:v>975</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="s">
-        <x:v>976</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" hidden="0" customHeight="1">
@@ -4701,13 +4695,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B7" s="11" t="s">
+        <x:v>975</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="s">
+        <x:v>976</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="s">
         <x:v>977</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="s">
-        <x:v>978</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="s">
-        <x:v>979</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" hidden="0" customHeight="1">
@@ -4715,13 +4709,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B8" s="11" t="s">
+        <x:v>978</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="s">
+        <x:v>979</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="s">
         <x:v>980</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="s">
-        <x:v>981</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="s">
-        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" hidden="0" customHeight="1">
@@ -4729,13 +4723,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B9" s="11" t="s">
-        <x:v>861</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="C9" s="11" t="s">
-        <x:v>983</x:v>
+        <x:v>981</x:v>
       </x:c>
       <x:c r="D9" s="11" t="s">
-        <x:v>984</x:v>
+        <x:v>982</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" hidden="0" customHeight="1">
@@ -4743,13 +4737,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B10" s="11" t="s">
-        <x:v>865</x:v>
+        <x:v>864</x:v>
       </x:c>
       <x:c r="C10" s="11" t="s">
-        <x:v>985</x:v>
+        <x:v>983</x:v>
       </x:c>
       <x:c r="D10" s="11" t="s">
-        <x:v>986</x:v>
+        <x:v>984</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" hidden="0" customHeight="1">
@@ -4757,13 +4751,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B11" s="11" t="s">
-        <x:v>857</x:v>
+        <x:v>856</x:v>
       </x:c>
       <x:c r="C11" s="11" t="s">
-        <x:v>987</x:v>
+        <x:v>985</x:v>
       </x:c>
       <x:c r="D11" s="11" t="s">
-        <x:v>988</x:v>
+        <x:v>986</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" hidden="0" customHeight="1">
@@ -4771,13 +4765,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B12" s="11" t="s">
+        <x:v>987</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="s">
+        <x:v>988</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="s">
         <x:v>989</x:v>
-      </x:c>
-      <x:c r="C12" s="11" t="s">
-        <x:v>990</x:v>
-      </x:c>
-      <x:c r="D12" s="11" t="s">
-        <x:v>991</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" hidden="0" customHeight="1">
@@ -4785,13 +4779,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B13" s="11" t="s">
+        <x:v>990</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="s">
+        <x:v>991</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="s">
         <x:v>992</x:v>
-      </x:c>
-      <x:c r="C13" s="11" t="s">
-        <x:v>993</x:v>
-      </x:c>
-      <x:c r="D13" s="11" t="s">
-        <x:v>994</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" hidden="0" customHeight="1">
@@ -4799,13 +4793,13 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="B14" s="11" t="s">
+        <x:v>993</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="s">
+        <x:v>994</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="s">
         <x:v>995</x:v>
-      </x:c>
-      <x:c r="C14" s="11" t="s">
-        <x:v>996</x:v>
-      </x:c>
-      <x:c r="D14" s="11" t="s">
-        <x:v>997</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -4899,7 +4893,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9cf40fe4fde48b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cf5eb4bc01b4748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5466,7 +5460,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ceaa622b814096"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9971dd92406c44b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13570,7 +13564,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra93a0139f9124430"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63b8dc4a0e144de3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14351,7 +14345,7 @@
     <x:mergeCell ref="I4:N4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa640940e73349db"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd35bb2711b64402c"/>
 </x:worksheet>
 </file>
 
@@ -14737,11 +14731,11 @@
       <x:c r="E18" s="11" t="s">
         <x:v>668</x:v>
       </x:c>
-      <x:c r="F18" s="12" t="s">
+      <x:c r="F18" s="12" t="str">
+        <x:v>Professional Dossier; https://www.eacmarkup.org/</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="s">
         <x:v>669</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="s">
-        <x:v>670</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="76" hidden="0" customHeight="1">
@@ -14749,13 +14743,13 @@
         <x:v>652</x:v>
       </x:c>
       <x:c r="B19" s="11" t="s">
+        <x:v>670</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="s">
         <x:v>671</x:v>
       </x:c>
-      <x:c r="C19" s="11" t="s">
+      <x:c r="D19" s="11" t="s">
         <x:v>672</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="s">
-        <x:v>673</x:v>
       </x:c>
       <x:c r="E19" s="11" t="s">
         <x:v>659</x:v>
@@ -14764,18 +14758,18 @@
         <x:v>611</x:v>
       </x:c>
       <x:c r="G19" s="11" t="s">
-        <x:v>674</x:v>
+        <x:v>673</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="76" hidden="0" customHeight="1">
       <x:c r="A20" s="11" t="s">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="s">
         <x:v>675</x:v>
       </x:c>
-      <x:c r="B20" s="11" t="s">
+      <x:c r="C20" s="11" t="s">
         <x:v>676</x:v>
-      </x:c>
-      <x:c r="C20" s="11" t="s">
-        <x:v>677</x:v>
       </x:c>
       <x:c r="D20" s="11" t="s">
         <x:v>655</x:v>
@@ -14787,67 +14781,67 @@
         <x:v>602</x:v>
       </x:c>
       <x:c r="G20" s="11" t="s">
-        <x:v>678</x:v>
+        <x:v>677</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="76" hidden="0" customHeight="1">
       <x:c r="A21" s="11" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="s">
         <x:v>679</x:v>
       </x:c>
-      <x:c r="B21" s="11" t="s">
+      <x:c r="C21" s="11" t="s">
         <x:v>680</x:v>
       </x:c>
-      <x:c r="C21" s="11" t="s">
+      <x:c r="D21" s="11" t="s">
         <x:v>681</x:v>
       </x:c>
-      <x:c r="D21" s="11" t="s">
+      <x:c r="E21" s="11" t="s">
         <x:v>682</x:v>
-      </x:c>
-      <x:c r="E21" s="11" t="s">
-        <x:v>683</x:v>
       </x:c>
       <x:c r="F21" s="12" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="G21" s="11" t="s">
-        <x:v>684</x:v>
+        <x:v>683</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="76" hidden="0" customHeight="1">
       <x:c r="A22" s="11" t="s">
+        <x:v>684</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="s">
         <x:v>685</x:v>
       </x:c>
-      <x:c r="B22" s="11" t="s">
+      <x:c r="C22" s="11" t="s">
         <x:v>686</x:v>
       </x:c>
-      <x:c r="C22" s="11" t="s">
+      <x:c r="D22" s="11" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="D22" s="11" t="s">
+      <x:c r="E22" s="11" t="s">
         <x:v>688</x:v>
       </x:c>
-      <x:c r="E22" s="11" t="s">
+      <x:c r="F22" s="12" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="F22" s="12" t="s">
+      <x:c r="G22" s="11" t="s">
         <x:v>690</x:v>
-      </x:c>
-      <x:c r="G22" s="11" t="s">
-        <x:v>691</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="76" hidden="0" customHeight="1">
       <x:c r="A23" s="11" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="s">
         <x:v>692</x:v>
       </x:c>
-      <x:c r="B23" s="11" t="s">
+      <x:c r="C23" s="11" t="s">
         <x:v>693</x:v>
       </x:c>
-      <x:c r="C23" s="11" t="s">
-        <x:v>694</x:v>
-      </x:c>
       <x:c r="D23" s="11" t="s">
-        <x:v>673</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="E23" s="11" t="s">
         <x:v>636</x:v>
@@ -14856,18 +14850,18 @@
         <x:v>611</x:v>
       </x:c>
       <x:c r="G23" s="11" t="s">
-        <x:v>695</x:v>
+        <x:v>694</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="76" hidden="0" customHeight="1">
       <x:c r="A24" s="11" t="s">
-        <x:v>692</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="B24" s="11" t="s">
+        <x:v>695</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="s">
         <x:v>696</x:v>
-      </x:c>
-      <x:c r="C24" s="11" t="s">
-        <x:v>697</x:v>
       </x:c>
       <x:c r="D24" s="11" t="s">
         <x:v>655</x:v>
@@ -14879,142 +14873,142 @@
         <x:v>602</x:v>
       </x:c>
       <x:c r="G24" s="11" t="s">
-        <x:v>698</x:v>
+        <x:v>697</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="76" hidden="0" customHeight="1">
       <x:c r="A25" s="11" t="s">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="s">
         <x:v>699</x:v>
       </x:c>
-      <x:c r="B25" s="11" t="s">
+      <x:c r="C25" s="11" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="C25" s="11" t="s">
+      <x:c r="D25" s="11" t="s">
         <x:v>701</x:v>
       </x:c>
-      <x:c r="D25" s="11" t="s">
+      <x:c r="E25" s="11" t="s">
         <x:v>702</x:v>
       </x:c>
-      <x:c r="E25" s="11" t="s">
+      <x:c r="F25" s="12" t="s">
         <x:v>703</x:v>
       </x:c>
-      <x:c r="F25" s="12" t="s">
+      <x:c r="G25" s="11" t="s">
         <x:v>704</x:v>
-      </x:c>
-      <x:c r="G25" s="11" t="s">
-        <x:v>705</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="76" hidden="0" customHeight="1">
       <x:c r="A26" s="11" t="s">
-        <x:v>699</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="B26" s="11" t="s">
+        <x:v>705</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="s">
         <x:v>706</x:v>
       </x:c>
-      <x:c r="C26" s="11" t="s">
+      <x:c r="D26" s="11" t="s">
+        <x:v>701</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="F26" s="12" t="s">
         <x:v>707</x:v>
       </x:c>
-      <x:c r="D26" s="11" t="s">
-        <x:v>702</x:v>
-      </x:c>
-      <x:c r="E26" s="11" t="s">
-        <x:v>703</x:v>
-      </x:c>
-      <x:c r="F26" s="12" t="s">
+      <x:c r="G26" s="11" t="s">
         <x:v>708</x:v>
-      </x:c>
-      <x:c r="G26" s="11" t="s">
-        <x:v>709</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="76" hidden="0" customHeight="1">
       <x:c r="A27" s="11" t="s">
+        <x:v>709</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="s">
         <x:v>710</x:v>
       </x:c>
-      <x:c r="B27" s="11" t="s">
+      <x:c r="C27" s="11" t="s">
         <x:v>711</x:v>
       </x:c>
-      <x:c r="C27" s="11" t="s">
+      <x:c r="D27" s="11" t="s">
         <x:v>712</x:v>
       </x:c>
-      <x:c r="D27" s="11" t="s">
+      <x:c r="E27" s="11" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="F27" s="12" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="s">
         <x:v>713</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="s">
-        <x:v>703</x:v>
-      </x:c>
-      <x:c r="F27" s="12" t="s">
-        <x:v>708</x:v>
-      </x:c>
-      <x:c r="G27" s="11" t="s">
-        <x:v>714</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="76" hidden="0" customHeight="1">
       <x:c r="A28" s="11" t="s">
+        <x:v>714</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="s">
         <x:v>715</x:v>
       </x:c>
-      <x:c r="B28" s="11" t="s">
+      <x:c r="C28" s="11" t="s">
         <x:v>716</x:v>
       </x:c>
-      <x:c r="C28" s="11" t="s">
+      <x:c r="D28" s="11" t="s">
         <x:v>717</x:v>
       </x:c>
-      <x:c r="D28" s="11" t="s">
+      <x:c r="E28" s="11" t="s">
         <x:v>718</x:v>
       </x:c>
-      <x:c r="E28" s="11" t="s">
+      <x:c r="F28" s="12" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="G28" s="11" t="s">
         <x:v>719</x:v>
-      </x:c>
-      <x:c r="F28" s="12" t="s">
-        <x:v>708</x:v>
-      </x:c>
-      <x:c r="G28" s="11" t="s">
-        <x:v>720</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="76" hidden="0" customHeight="1">
       <x:c r="A29" s="11" t="s">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="s">
         <x:v>721</x:v>
       </x:c>
-      <x:c r="B29" s="11" t="s">
+      <x:c r="C29" s="11" t="s">
         <x:v>722</x:v>
       </x:c>
-      <x:c r="C29" s="11" t="s">
+      <x:c r="D29" s="11" t="s">
         <x:v>723</x:v>
       </x:c>
-      <x:c r="D29" s="11" t="s">
+      <x:c r="E29" s="11" t="s">
+        <x:v>718</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="G29" s="11" t="s">
         <x:v>724</x:v>
-      </x:c>
-      <x:c r="E29" s="11" t="s">
-        <x:v>719</x:v>
-      </x:c>
-      <x:c r="F29" s="12" t="s">
-        <x:v>708</x:v>
-      </x:c>
-      <x:c r="G29" s="11" t="s">
-        <x:v>725</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="76" hidden="0" customHeight="1">
       <x:c r="A30" s="11" t="s">
-        <x:v>726</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="B30" s="11" t="str">
         <x:v>Supplied archive: 444 distinct audio records, approximately 249.67 hours, 2021–2025; 437 are at least twenty minutes.</x:v>
       </x:c>
       <x:c r="C30" s="11" t="s">
+        <x:v>726</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="s">
         <x:v>727</x:v>
       </x:c>
-      <x:c r="D30" s="11" t="s">
+      <x:c r="E30" s="11" t="s">
         <x:v>728</x:v>
       </x:c>
-      <x:c r="E30" s="11" t="s">
+      <x:c r="F30" s="12" t="s">
         <x:v>729</x:v>
-      </x:c>
-      <x:c r="F30" s="12" t="s">
-        <x:v>730</x:v>
       </x:c>
       <x:c r="G30" s="11" t="str">
         <x:v>The audio messages are separate from the YouTube messages, as confirmed by the source owner.</x:v>
@@ -15022,7 +15016,7 @@
     </x:row>
     <x:row r="31" ht="76" hidden="0" customHeight="1">
       <x:c r="A31" s="11" t="s">
-        <x:v>726</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="B31" s="11" t="str">
         <x:v>Public Brother Llewellyn playlist on the church channel on YouTube: 387 videos, approximately 438.86 hours, visible dates 2018–2023.</x:v>
@@ -15031,13 +15025,13 @@
         <x:v>Use as additive evidence of sustained public communication and long-form teaching.</x:v>
       </x:c>
       <x:c r="D31" s="11" t="s">
+        <x:v>730</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="s">
         <x:v>731</x:v>
       </x:c>
-      <x:c r="E31" s="11" t="s">
+      <x:c r="F31" s="12" t="s">
         <x:v>732</x:v>
-      </x:c>
-      <x:c r="F31" s="12" t="s">
-        <x:v>733</x:v>
       </x:c>
       <x:c r="G31" s="11" t="str">
         <x:v>Additive with the supplied archive: approximately 831 sermons and 688.53 hours (approximately 689) across 8 years.</x:v>
@@ -15045,13 +15039,13 @@
     </x:row>
     <x:row r="32" ht="76" hidden="0" customHeight="1">
       <x:c r="A32" s="11" t="s">
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="s">
         <x:v>734</x:v>
       </x:c>
-      <x:c r="B32" s="11" t="s">
+      <x:c r="C32" s="11" t="s">
         <x:v>735</x:v>
-      </x:c>
-      <x:c r="C32" s="11" t="s">
-        <x:v>736</x:v>
       </x:c>
       <x:c r="D32" s="11" t="s">
         <x:v>600</x:v>
@@ -15063,18 +15057,18 @@
         <x:v>602</x:v>
       </x:c>
       <x:c r="G32" s="11" t="s">
-        <x:v>737</x:v>
+        <x:v>736</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="76" hidden="0" customHeight="1">
       <x:c r="A33" s="11" t="s">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="s">
         <x:v>738</x:v>
       </x:c>
-      <x:c r="B33" s="11" t="s">
+      <x:c r="C33" s="11" t="s">
         <x:v>739</x:v>
-      </x:c>
-      <x:c r="C33" s="11" t="s">
-        <x:v>740</x:v>
       </x:c>
       <x:c r="D33" s="11" t="s">
         <x:v>600</x:v>
@@ -15083,21 +15077,21 @@
         <x:v>601</x:v>
       </x:c>
       <x:c r="F33" s="12" t="s">
+        <x:v>740</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="s">
         <x:v>741</x:v>
-      </x:c>
-      <x:c r="G33" s="11" t="s">
-        <x:v>742</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="76" hidden="0" customHeight="1">
       <x:c r="A34" s="11" t="s">
-        <x:v>738</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="B34" s="11" t="s">
+        <x:v>742</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="s">
         <x:v>743</x:v>
-      </x:c>
-      <x:c r="C34" s="11" t="s">
-        <x:v>744</x:v>
       </x:c>
       <x:c r="D34" s="11" t="s">
         <x:v>600</x:v>
@@ -15109,18 +15103,18 @@
         <x:v>602</x:v>
       </x:c>
       <x:c r="G34" s="11" t="s">
-        <x:v>745</x:v>
+        <x:v>744</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="76" hidden="0" customHeight="1">
       <x:c r="A35" s="11" t="s">
+        <x:v>745</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="s">
         <x:v>746</x:v>
       </x:c>
-      <x:c r="B35" s="11" t="s">
+      <x:c r="C35" s="11" t="s">
         <x:v>747</x:v>
-      </x:c>
-      <x:c r="C35" s="11" t="s">
-        <x:v>748</x:v>
       </x:c>
       <x:c r="D35" s="11" t="s">
         <x:v>600</x:v>
@@ -15129,21 +15123,21 @@
         <x:v>601</x:v>
       </x:c>
       <x:c r="F35" s="12" t="s">
+        <x:v>748</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="s">
         <x:v>749</x:v>
-      </x:c>
-      <x:c r="G35" s="11" t="s">
-        <x:v>750</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="76" hidden="0" customHeight="1">
       <x:c r="A36" s="11" t="s">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="s">
         <x:v>751</x:v>
       </x:c>
-      <x:c r="B36" s="11" t="s">
+      <x:c r="C36" s="11" t="s">
         <x:v>752</x:v>
-      </x:c>
-      <x:c r="C36" s="11" t="s">
-        <x:v>753</x:v>
       </x:c>
       <x:c r="D36" s="11" t="s">
         <x:v>655</x:v>
@@ -15152,21 +15146,21 @@
         <x:v>601</x:v>
       </x:c>
       <x:c r="F36" s="12" t="s">
+        <x:v>753</x:v>
+      </x:c>
+      <x:c r="G36" s="11" t="s">
         <x:v>754</x:v>
-      </x:c>
-      <x:c r="G36" s="11" t="s">
-        <x:v>755</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="76" hidden="0" customHeight="1">
       <x:c r="A37" s="11" t="s">
+        <x:v>755</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="s">
         <x:v>756</x:v>
       </x:c>
-      <x:c r="B37" s="11" t="s">
+      <x:c r="C37" s="11" t="s">
         <x:v>757</x:v>
-      </x:c>
-      <x:c r="C37" s="11" t="s">
-        <x:v>758</x:v>
       </x:c>
       <x:c r="D37" s="11" t="s">
         <x:v>655</x:v>
@@ -15175,10 +15169,10 @@
         <x:v>601</x:v>
       </x:c>
       <x:c r="F37" s="12" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="G37" s="11" t="s">
         <x:v>759</x:v>
-      </x:c>
-      <x:c r="G37" s="11" t="s">
-        <x:v>760</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="68" customHeight="1">
@@ -15251,7 +15245,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0269e33adeb54873"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdebcfbc647cc489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15270,7 +15264,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>761</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -15298,7 +15292,7 @@
     </x:row>
     <x:row r="4" ht="30" hidden="0" customHeight="1">
       <x:c r="A4" s="13" t="s">
-        <x:v>762</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="B4" s="13"/>
       <x:c r="C4" s="13"/>
@@ -15308,182 +15302,182 @@
     </x:row>
     <x:row r="5" ht="30" hidden="0" customHeight="1">
       <x:c r="A5" s="15" t="s">
+        <x:v>762</x:v>
+      </x:c>
+      <x:c r="B5" s="15" t="s">
         <x:v>763</x:v>
       </x:c>
-      <x:c r="B5" s="15" t="s">
+      <x:c r="C5" s="15" t="s">
         <x:v>764</x:v>
       </x:c>
-      <x:c r="C5" s="15" t="s">
+      <x:c r="D5" s="15" t="s">
         <x:v>765</x:v>
       </x:c>
-      <x:c r="D5" s="15" t="s">
+      <x:c r="E5" s="15" t="s">
         <x:v>766</x:v>
       </x:c>
-      <x:c r="E5" s="15" t="s">
+      <x:c r="F5" s="15" t="s">
         <x:v>767</x:v>
-      </x:c>
-      <x:c r="F5" s="15" t="s">
-        <x:v>768</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" hidden="0" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>769</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="B6" s="30" t="n">
         <x:v>268</x:v>
       </x:c>
       <x:c r="C6" s="11" t="s">
+        <x:v>769</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="s">
         <x:v>770</x:v>
       </x:c>
-      <x:c r="D6" s="11" t="s">
+      <x:c r="E6" s="11" t="s">
         <x:v>771</x:v>
       </x:c>
-      <x:c r="E6" s="11" t="s">
+      <x:c r="F6" s="11" t="s">
         <x:v>772</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="s">
-        <x:v>773</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>774</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="B7" s="30" t="n">
         <x:v>141</x:v>
       </x:c>
       <x:c r="C7" s="11" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="s">
         <x:v>775</x:v>
       </x:c>
-      <x:c r="D7" s="11" t="s">
+      <x:c r="E7" s="11" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="s">
         <x:v>776</x:v>
-      </x:c>
-      <x:c r="E7" s="11" t="s">
-        <x:v>772</x:v>
-      </x:c>
-      <x:c r="F7" s="11" t="s">
-        <x:v>777</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" hidden="0" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>778</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="B8" s="30" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="11" t="s">
+        <x:v>778</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="s">
         <x:v>779</x:v>
       </x:c>
-      <x:c r="D8" s="11" t="s">
+      <x:c r="E8" s="11" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="s">
         <x:v>780</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="s">
-        <x:v>772</x:v>
-      </x:c>
-      <x:c r="F8" s="11" t="s">
-        <x:v>781</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" hidden="0" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>782</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="B9" s="30" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="C9" s="11" t="s">
+        <x:v>782</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="s">
         <x:v>783</x:v>
       </x:c>
-      <x:c r="D9" s="11" t="s">
+      <x:c r="E9" s="11" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="s">
         <x:v>784</x:v>
-      </x:c>
-      <x:c r="E9" s="11" t="s">
-        <x:v>772</x:v>
-      </x:c>
-      <x:c r="F9" s="11" t="s">
-        <x:v>785</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" hidden="0" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>786</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
         <x:v>104</x:v>
       </x:c>
       <x:c r="C10" s="11" t="s">
+        <x:v>786</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="s">
         <x:v>787</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="s">
+      <x:c r="E10" s="11" t="s">
         <x:v>788</x:v>
       </x:c>
-      <x:c r="E10" s="11" t="s">
+      <x:c r="F10" s="11" t="s">
         <x:v>789</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="s">
-        <x:v>790</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" hidden="0" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>791</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="B11" s="30" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="11" t="s">
+        <x:v>791</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="s">
         <x:v>792</x:v>
       </x:c>
-      <x:c r="D11" s="11" t="s">
+      <x:c r="E11" s="11" t="s">
+        <x:v>788</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="s">
         <x:v>793</x:v>
-      </x:c>
-      <x:c r="E11" s="11" t="s">
-        <x:v>789</x:v>
-      </x:c>
-      <x:c r="F11" s="11" t="s">
-        <x:v>794</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" hidden="0" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>795</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="B12" s="30" t="n">
         <x:v>109</x:v>
       </x:c>
       <x:c r="C12" s="11" t="s">
+        <x:v>795</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="s">
         <x:v>796</x:v>
       </x:c>
-      <x:c r="D12" s="11" t="s">
+      <x:c r="E12" s="11" t="s">
+        <x:v>788</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="s">
         <x:v>797</x:v>
-      </x:c>
-      <x:c r="E12" s="11" t="s">
-        <x:v>789</x:v>
-      </x:c>
-      <x:c r="F12" s="11" t="s">
-        <x:v>798</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" hidden="0" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>799</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="B13" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="11" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="D13" s="11" t="s">
+      <x:c r="E13" s="11" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="s">
         <x:v>801</x:v>
-      </x:c>
-      <x:c r="E13" s="11" t="s">
-        <x:v>772</x:v>
-      </x:c>
-      <x:c r="F13" s="11" t="s">
-        <x:v>802</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
@@ -15504,7 +15498,7 @@
     </x:row>
     <x:row r="16" ht="30" hidden="0" customHeight="1">
       <x:c r="A16" s="29" t="s">
-        <x:v>803</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="B16" s="29"/>
       <x:c r="C16" s="29"/>
@@ -15520,10 +15514,10 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="C17" s="15" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="D17" s="15" t="s">
         <x:v>804</x:v>
-      </x:c>
-      <x:c r="D17" s="15" t="s">
-        <x:v>805</x:v>
       </x:c>
       <x:c r="E17" s="15" t="s">
         <x:v>124</x:v>
@@ -15657,7 +15651,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>806</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -15691,33 +15685,33 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="15" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
+        <x:v>763</x:v>
+      </x:c>
+      <x:c r="C4" s="15" t="s">
         <x:v>807</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
-        <x:v>764</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
+      <x:c r="D4" s="15" t="s">
         <x:v>808</x:v>
       </x:c>
-      <x:c r="D4" s="15" t="s">
+      <x:c r="E4" s="15" t="s">
         <x:v>809</x:v>
       </x:c>
-      <x:c r="E4" s="15" t="s">
+      <x:c r="F4" s="15" t="s">
         <x:v>810</x:v>
       </x:c>
-      <x:c r="F4" s="15" t="s">
+      <x:c r="G4" s="15" t="s">
         <x:v>811</x:v>
       </x:c>
-      <x:c r="G4" s="15" t="s">
+      <x:c r="H4" s="15" t="s">
         <x:v>812</x:v>
-      </x:c>
-      <x:c r="H4" s="15" t="s">
-        <x:v>813</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="68" hidden="0" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>814</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="B5" s="31" t="n">
         <x:v>444</x:v>
@@ -15735,7 +15729,7 @@
         <x:v>Distinct audio recordings within the supplied archive; 437 recordings are at least twenty minutes. These messages are separate from the public YouTube playlist.</x:v>
       </x:c>
       <x:c r="G5" s="12" t="s">
-        <x:v>815</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
         <x:v>High within supplied archive; distinct from playlist confirmed by source owner</x:v>
@@ -15743,7 +15737,7 @@
     </x:row>
     <x:row r="6" ht="68" hidden="0" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>816</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="B6" s="31" t="n">
         <x:v>387</x:v>
@@ -15761,7 +15755,7 @@
         <x:v>Unique public Brother Llewellyn playlist videos on the church channel. These messages are separate from the supplied audio archive; duration uses displayed rounded labels.</x:v>
       </x:c>
       <x:c r="G6" s="12" t="s">
-        <x:v>733</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="H6" s="11" t="str">
         <x:v>High as of original audit date; distinct from archive confirmed by source owner</x:v>
@@ -15809,7 +15803,7 @@
     </x:row>
     <x:row r="9" ht="28" hidden="0" customHeight="1">
       <x:c r="A9" s="29" t="s">
-        <x:v>817</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="B9" s="29"/>
       <x:c r="C9" s="29"/>
@@ -15821,16 +15815,16 @@
     </x:row>
     <x:row r="10" ht="28" hidden="0" customHeight="1">
       <x:c r="A10" s="15" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="s">
         <x:v>818</x:v>
       </x:c>
-      <x:c r="B10" s="15" t="s">
+      <x:c r="C10" s="15" t="s">
+        <x:v>807</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="s">
         <x:v>819</x:v>
-      </x:c>
-      <x:c r="C10" s="15" t="s">
-        <x:v>808</x:v>
-      </x:c>
-      <x:c r="D10" s="15" t="s">
-        <x:v>820</x:v>
       </x:c>
       <x:c r="E10" s="3"/>
       <x:c r="F10" s="3"/>
@@ -15848,7 +15842,7 @@
         <x:v>2.02</x:v>
       </x:c>
       <x:c r="D11" s="11" t="s">
-        <x:v>821</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="E11" s="3"/>
       <x:c r="F11" s="3"/>
@@ -15866,7 +15860,7 @@
         <x:v>13.69</x:v>
       </x:c>
       <x:c r="D12" s="11" t="s">
-        <x:v>822</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="E12" s="3"/>
       <x:c r="F12" s="3"/>
@@ -15884,7 +15878,7 @@
         <x:v>74.92</x:v>
       </x:c>
       <x:c r="D13" s="11" t="s">
-        <x:v>823</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="E13" s="3"/>
       <x:c r="F13" s="3"/>
@@ -15902,7 +15896,7 @@
         <x:v>77.43</x:v>
       </x:c>
       <x:c r="D14" s="11" t="s">
-        <x:v>824</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="E14" s="3"/>
       <x:c r="F14" s="3"/>
@@ -15920,7 +15914,7 @@
         <x:v>81.61</x:v>
       </x:c>
       <x:c r="D15" s="11" t="s">
-        <x:v>825</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="E15" s="3"/>
       <x:c r="F15" s="3"/>
@@ -15951,7 +15945,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>826</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -15961,7 +15955,7 @@
     </x:row>
     <x:row r="2" ht="30" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>827</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -15979,33 +15973,33 @@
     </x:row>
     <x:row r="4" ht="32" hidden="0" customHeight="1">
       <x:c r="A4" s="15" t="s">
+        <x:v>827</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="s">
+        <x:v>811</x:v>
+      </x:c>
+      <x:c r="C4" s="15" t="s">
         <x:v>828</x:v>
       </x:c>
-      <x:c r="B4" s="15" t="s">
-        <x:v>812</x:v>
-      </x:c>
-      <x:c r="C4" s="15" t="s">
+      <x:c r="D4" s="15" t="s">
         <x:v>829</x:v>
       </x:c>
-      <x:c r="D4" s="15" t="s">
+      <x:c r="E4" s="15" t="s">
         <x:v>830</x:v>
       </x:c>
-      <x:c r="E4" s="15" t="s">
+      <x:c r="F4" s="15" t="s">
         <x:v>831</x:v>
-      </x:c>
-      <x:c r="F4" s="15" t="s">
-        <x:v>832</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="52" hidden="0" customHeight="1">
       <x:c r="A5" s="11" t="s">
+        <x:v>832</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="s">
         <x:v>833</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="s">
+      <x:c r="C5" s="11" t="s">
         <x:v>834</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="s">
-        <x:v>835</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>Llewellyn_van_der_Merwe_Executive_CV.pdf</x:v>
@@ -16019,13 +16013,13 @@
     </x:row>
     <x:row r="6" ht="52" hidden="0" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>833</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="B6" s="11" t="s">
-        <x:v>708</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="C6" s="11" t="s">
-        <x:v>836</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
         <x:v>Llewellyn_van_der_Merwe_Professional_Dossier.pdf</x:v>
@@ -16034,12 +16028,12 @@
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F6" s="11" t="s">
-        <x:v>837</x:v>
+        <x:v>836</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>833</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
         <x:v>Canonical Evidence Ledger — 28 July baseline</x:v>
@@ -16062,10 +16056,10 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="B8" s="11" t="s">
+        <x:v>837</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="s">
         <x:v>838</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="s">
-        <x:v>839</x:v>
       </x:c>
       <x:c r="D8" s="12" t="s">
         <x:v>602</x:v>
@@ -16074,7 +16068,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F8" s="11" t="s">
-        <x:v>840</x:v>
+        <x:v>839</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="52" hidden="0" customHeight="1">
@@ -16082,19 +16076,19 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="B9" s="11" t="s">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="s">
         <x:v>841</x:v>
       </x:c>
-      <x:c r="C9" s="11" t="s">
+      <x:c r="D9" s="12" t="s">
         <x:v>842</x:v>
-      </x:c>
-      <x:c r="D9" s="12" t="s">
-        <x:v>843</x:v>
       </x:c>
       <x:c r="E9" s="17" t="n">
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F9" s="11" t="s">
-        <x:v>844</x:v>
+        <x:v>843</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="52" hidden="0" customHeight="1">
@@ -16105,7 +16099,7 @@
         <x:v>Production master prompt source</x:v>
       </x:c>
       <x:c r="C10" s="11" t="s">
-        <x:v>845</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Pasted markdown.md</x:v>
@@ -16119,16 +16113,16 @@
     </x:row>
     <x:row r="11" ht="52" hidden="0" customHeight="1">
       <x:c r="A11" s="11" t="s">
+        <x:v>845</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="s">
         <x:v>846</x:v>
       </x:c>
-      <x:c r="B11" s="11" t="s">
+      <x:c r="C11" s="11" t="s">
         <x:v>847</x:v>
       </x:c>
-      <x:c r="C11" s="11" t="s">
-        <x:v>848</x:v>
-      </x:c>
       <x:c r="D11" s="12" t="s">
-        <x:v>749</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="E11" s="33" t="n">
         <x:v>46232</x:v>
@@ -16139,16 +16133,16 @@
     </x:row>
     <x:row r="12" ht="52" hidden="0" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>846</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="B12" s="11" t="s">
+        <x:v>848</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="s">
         <x:v>849</x:v>
       </x:c>
-      <x:c r="C12" s="11" t="s">
+      <x:c r="D12" s="12" t="s">
         <x:v>850</x:v>
-      </x:c>
-      <x:c r="D12" s="12" t="s">
-        <x:v>851</x:v>
       </x:c>
       <x:c r="E12" s="33" t="n">
         <x:v>46232</x:v>
@@ -16159,13 +16153,13 @@
     </x:row>
     <x:row r="13" ht="52" hidden="0" customHeight="1">
       <x:c r="A13" s="11" t="s">
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="s">
         <x:v>852</x:v>
       </x:c>
-      <x:c r="B13" s="11" t="s">
+      <x:c r="C13" s="11" t="s">
         <x:v>853</x:v>
-      </x:c>
-      <x:c r="C13" s="11" t="s">
-        <x:v>854</x:v>
       </x:c>
       <x:c r="D13" s="12" t="s">
         <x:v>630</x:v>
@@ -16174,107 +16168,107 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F13" s="11" t="s">
-        <x:v>855</x:v>
+        <x:v>854</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="52" hidden="0" customHeight="1">
       <x:c r="A14" s="11" t="s">
+        <x:v>855</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="s">
         <x:v>856</x:v>
       </x:c>
-      <x:c r="B14" s="11" t="s">
+      <x:c r="C14" s="11" t="s">
         <x:v>857</x:v>
       </x:c>
-      <x:c r="C14" s="11" t="s">
+      <x:c r="D14" s="12" t="s">
         <x:v>858</x:v>
-      </x:c>
-      <x:c r="D14" s="12" t="s">
-        <x:v>859</x:v>
       </x:c>
       <x:c r="E14" s="33" t="n">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F14" s="11" t="s">
-        <x:v>860</x:v>
+        <x:v>859</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52" hidden="0" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>856</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="B15" s="11" t="s">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="s">
         <x:v>861</x:v>
       </x:c>
-      <x:c r="C15" s="11" t="s">
+      <x:c r="D15" s="12" t="s">
         <x:v>862</x:v>
-      </x:c>
-      <x:c r="D15" s="12" t="s">
-        <x:v>863</x:v>
       </x:c>
       <x:c r="E15" s="33" t="n">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F15" s="11" t="s">
-        <x:v>864</x:v>
+        <x:v>863</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" hidden="0" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>856</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="B16" s="11" t="s">
+        <x:v>864</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="s">
         <x:v>865</x:v>
       </x:c>
-      <x:c r="C16" s="11" t="s">
+      <x:c r="D16" s="12" t="s">
         <x:v>866</x:v>
-      </x:c>
-      <x:c r="D16" s="12" t="s">
-        <x:v>867</x:v>
       </x:c>
       <x:c r="E16" s="33" t="n">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F16" s="11" t="s">
-        <x:v>868</x:v>
+        <x:v>867</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="52" hidden="0" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>856</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="B17" s="11" t="s">
+        <x:v>868</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="s">
         <x:v>869</x:v>
       </x:c>
-      <x:c r="C17" s="11" t="s">
+      <x:c r="D17" s="12" t="s">
         <x:v>870</x:v>
-      </x:c>
-      <x:c r="D17" s="12" t="s">
-        <x:v>871</x:v>
       </x:c>
       <x:c r="E17" s="17" t="n">
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F17" s="11" t="s">
-        <x:v>872</x:v>
+        <x:v>871</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="52" hidden="0" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>856</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="B18" s="11" t="s">
+        <x:v>872</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="s">
         <x:v>873</x:v>
       </x:c>
-      <x:c r="C18" s="11" t="s">
+      <x:c r="D18" s="12" t="s">
         <x:v>874</x:v>
-      </x:c>
-      <x:c r="D18" s="12" t="s">
-        <x:v>875</x:v>
       </x:c>
       <x:c r="E18" s="17" t="n">
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F18" s="11" t="s">
-        <x:v>876</x:v>
+        <x:v>875</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="52" hidden="0" customHeight="1">
@@ -16282,10 +16276,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B19" s="11" t="s">
+        <x:v>876</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="s">
         <x:v>877</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="s">
-        <x:v>878</x:v>
       </x:c>
       <x:c r="D19" s="12" t="s">
         <x:v>18</x:v>
@@ -16294,7 +16288,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F19" s="11" t="s">
-        <x:v>879</x:v>
+        <x:v>878</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="52" hidden="0" customHeight="1">
@@ -16302,10 +16296,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B20" s="11" t="s">
+        <x:v>879</x:v>
+      </x:c>
+      <x:c r="C20" s="11" t="s">
         <x:v>880</x:v>
-      </x:c>
-      <x:c r="C20" s="11" t="s">
-        <x:v>881</x:v>
       </x:c>
       <x:c r="D20" s="12" t="s">
         <x:v>23</x:v>
@@ -16322,10 +16316,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B21" s="11" t="s">
+        <x:v>881</x:v>
+      </x:c>
+      <x:c r="C21" s="11" t="s">
         <x:v>882</x:v>
-      </x:c>
-      <x:c r="C21" s="11" t="s">
-        <x:v>883</x:v>
       </x:c>
       <x:c r="D21" s="12" t="s">
         <x:v>27</x:v>
@@ -16334,7 +16328,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F21" s="11" t="s">
-        <x:v>884</x:v>
+        <x:v>883</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="52" hidden="0" customHeight="1">
@@ -16342,10 +16336,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B22" s="11" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="s">
         <x:v>885</x:v>
-      </x:c>
-      <x:c r="C22" s="11" t="s">
-        <x:v>886</x:v>
       </x:c>
       <x:c r="D22" s="12" t="s">
         <x:v>32</x:v>
@@ -16354,7 +16348,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F22" s="11" t="s">
-        <x:v>887</x:v>
+        <x:v>886</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="52" hidden="0" customHeight="1">
@@ -16362,10 +16356,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B23" s="11" t="s">
+        <x:v>887</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="s">
         <x:v>888</x:v>
-      </x:c>
-      <x:c r="C23" s="11" t="s">
-        <x:v>889</x:v>
       </x:c>
       <x:c r="D23" s="12" t="s">
         <x:v>38</x:v>
@@ -16374,7 +16368,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F23" s="11" t="s">
-        <x:v>890</x:v>
+        <x:v>889</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="52" hidden="0" customHeight="1">
@@ -16382,10 +16376,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B24" s="11" t="s">
+        <x:v>890</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="s">
         <x:v>891</x:v>
-      </x:c>
-      <x:c r="C24" s="11" t="s">
-        <x:v>892</x:v>
       </x:c>
       <x:c r="D24" s="12" t="s">
         <x:v>44</x:v>
@@ -16394,7 +16388,7 @@
         <x:v>46231</x:v>
       </x:c>
       <x:c r="F24" s="11" t="s">
-        <x:v>893</x:v>
+        <x:v>892</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="52" hidden="0" customHeight="1">
@@ -16402,10 +16396,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B25" s="11" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="s">
         <x:v>894</x:v>
-      </x:c>
-      <x:c r="C25" s="11" t="s">
-        <x:v>895</x:v>
       </x:c>
       <x:c r="D25" s="12" t="s">
         <x:v>47</x:v>
@@ -16422,10 +16416,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B26" s="11" t="s">
+        <x:v>895</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="s">
         <x:v>896</x:v>
-      </x:c>
-      <x:c r="C26" s="11" t="s">
-        <x:v>897</x:v>
       </x:c>
       <x:c r="D26" s="12" t="s">
         <x:v>52</x:v>
@@ -16434,7 +16428,7 @@
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F26" s="11" t="s">
-        <x:v>898</x:v>
+        <x:v>897</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="52" hidden="0" customHeight="1">
@@ -16442,10 +16436,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B27" s="11" t="s">
+        <x:v>898</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="C27" s="11" t="s">
-        <x:v>900</x:v>
       </x:c>
       <x:c r="D27" s="12" t="s">
         <x:v>57</x:v>
@@ -16454,7 +16448,7 @@
         <x:v>46232</x:v>
       </x:c>
       <x:c r="F27" s="11" t="s">
-        <x:v>901</x:v>
+        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="52" hidden="0" customHeight="1">
@@ -16462,10 +16456,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B28" s="11" t="s">
+        <x:v>901</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="s">
         <x:v>902</x:v>
-      </x:c>
-      <x:c r="C28" s="11" t="s">
-        <x:v>903</x:v>
       </x:c>
       <x:c r="D28" s="12" t="s">
         <x:v>62</x:v>
@@ -16482,10 +16476,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B29" s="11" t="s">
+        <x:v>903</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="s">
         <x:v>904</x:v>
-      </x:c>
-      <x:c r="C29" s="11" t="s">
-        <x:v>905</x:v>
       </x:c>
       <x:c r="D29" s="12" t="s">
         <x:v>66</x:v>
@@ -16499,96 +16493,96 @@
     </x:row>
     <x:row r="30" ht="52" hidden="0" customHeight="1">
       <x:c r="A30" s="11" t="s">
+        <x:v>905</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="s">
         <x:v>906</x:v>
       </x:c>
-      <x:c r="B30" s="11" t="s">
+      <x:c r="C30" s="11" t="s">
         <x:v>907</x:v>
       </x:c>
-      <x:c r="C30" s="11" t="s">
-        <x:v>908</x:v>
-      </x:c>
       <x:c r="D30" s="12" t="s">
-        <x:v>690</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="E30" s="17" t="n">
         <x:v>46221</x:v>
       </x:c>
       <x:c r="F30" s="11" t="s">
-        <x:v>909</x:v>
+        <x:v>908</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="52" hidden="0" customHeight="1">
       <x:c r="A31" s="11" t="s">
+        <x:v>909</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="s">
         <x:v>910</x:v>
       </x:c>
-      <x:c r="B31" s="11" t="s">
+      <x:c r="C31" s="11" t="s">
         <x:v>911</x:v>
       </x:c>
-      <x:c r="C31" s="11" t="s">
+      <x:c r="D31" s="12" t="s">
         <x:v>912</x:v>
-      </x:c>
-      <x:c r="D31" s="12" t="s">
-        <x:v>913</x:v>
       </x:c>
       <x:c r="E31" s="17" t="n">
         <x:v>46221</x:v>
       </x:c>
       <x:c r="F31" s="11" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="52" hidden="0" customHeight="1">
       <x:c r="A32" s="11" t="s">
-        <x:v>910</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="B32" s="11" t="s">
+        <x:v>914</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="s">
         <x:v>915</x:v>
       </x:c>
-      <x:c r="C32" s="11" t="s">
+      <x:c r="D32" s="12" t="s">
         <x:v>916</x:v>
-      </x:c>
-      <x:c r="D32" s="12" t="s">
-        <x:v>917</x:v>
       </x:c>
       <x:c r="E32" s="17" t="n">
         <x:v>46221</x:v>
       </x:c>
       <x:c r="F32" s="11" t="s">
-        <x:v>914</x:v>
+        <x:v>913</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="52" hidden="0" customHeight="1">
       <x:c r="A33" s="11" t="s">
+        <x:v>917</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="s">
         <x:v>918</x:v>
       </x:c>
-      <x:c r="B33" s="11" t="s">
+      <x:c r="C33" s="11" t="s">
         <x:v>919</x:v>
       </x:c>
-      <x:c r="C33" s="11" t="s">
-        <x:v>920</x:v>
-      </x:c>
-      <x:c r="D33" s="12" t="s">
-        <x:v>921</x:v>
+      <x:c r="D33" s="12" t="str">
+        <x:v>https://www.eacmarkup.org/</x:v>
       </x:c>
       <x:c r="E33" s="17" t="n">
         <x:v>46221</x:v>
       </x:c>
       <x:c r="F33" s="11" t="s">
-        <x:v>922</x:v>
+        <x:v>920</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="52" hidden="0" customHeight="1">
       <x:c r="A34" s="11" t="s">
+        <x:v>921</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="s">
+        <x:v>922</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="s">
         <x:v>923</x:v>
       </x:c>
-      <x:c r="B34" s="11" t="s">
-        <x:v>924</x:v>
-      </x:c>
-      <x:c r="C34" s="11" t="s">
-        <x:v>925</x:v>
-      </x:c>
       <x:c r="D34" s="12" t="s">
-        <x:v>733</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="E34" s="17" t="n">
         <x:v>46221</x:v>
@@ -16784,7 +16778,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e61382fb68b45c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59445f3903e64241"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16799,13 +16793,13 @@
   <x:sheetData>
     <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="s">
-        <x:v>926</x:v>
+        <x:v>924</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
     </x:row>
     <x:row r="2" ht="30" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>927</x:v>
+        <x:v>925</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
     </x:row>
@@ -16815,159 +16809,159 @@
     </x:row>
     <x:row r="4" ht="30" hidden="0" customHeight="1">
       <x:c r="A4" s="15" t="s">
-        <x:v>928</x:v>
+        <x:v>926</x:v>
       </x:c>
       <x:c r="B4" s="15" t="s">
-        <x:v>929</x:v>
+        <x:v>927</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="62" hidden="0" customHeight="1">
       <x:c r="A5" s="11" t="s">
-        <x:v>930</x:v>
+        <x:v>928</x:v>
       </x:c>
       <x:c r="B5" s="11" t="s">
-        <x:v>931</x:v>
+        <x:v>929</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="62" hidden="0" customHeight="1">
       <x:c r="A6" s="11" t="s">
-        <x:v>932</x:v>
+        <x:v>930</x:v>
       </x:c>
       <x:c r="B6" s="11" t="s">
-        <x:v>933</x:v>
+        <x:v>931</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="s">
-        <x:v>934</x:v>
+        <x:v>932</x:v>
       </x:c>
       <x:c r="B7" s="11" t="s">
-        <x:v>935</x:v>
+        <x:v>933</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" hidden="0" customHeight="1">
       <x:c r="A8" s="11" t="s">
-        <x:v>936</x:v>
+        <x:v>934</x:v>
       </x:c>
       <x:c r="B8" s="11" t="s">
-        <x:v>937</x:v>
+        <x:v>935</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" hidden="0" customHeight="1">
       <x:c r="A9" s="11" t="s">
-        <x:v>938</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="B9" s="11" t="s">
-        <x:v>939</x:v>
+        <x:v>937</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="62" hidden="0" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>940</x:v>
+        <x:v>938</x:v>
       </x:c>
       <x:c r="B10" s="11" t="s">
-        <x:v>941</x:v>
+        <x:v>939</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" hidden="0" customHeight="1">
       <x:c r="A11" s="11" t="s">
-        <x:v>942</x:v>
+        <x:v>940</x:v>
       </x:c>
       <x:c r="B11" s="11" t="s">
-        <x:v>943</x:v>
+        <x:v>941</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" hidden="0" customHeight="1">
       <x:c r="A12" s="11" t="s">
-        <x:v>794</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="B12" s="11" t="s">
-        <x:v>944</x:v>
+        <x:v>942</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="62" hidden="0" customHeight="1">
       <x:c r="A13" s="11" t="s">
-        <x:v>945</x:v>
+        <x:v>943</x:v>
       </x:c>
       <x:c r="B13" s="11" t="s">
-        <x:v>946</x:v>
+        <x:v>944</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="62" hidden="0" customHeight="1">
       <x:c r="A14" s="11" t="s">
-        <x:v>947</x:v>
+        <x:v>945</x:v>
       </x:c>
       <x:c r="B14" s="11" t="s">
-        <x:v>948</x:v>
+        <x:v>946</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="62" hidden="0" customHeight="1">
       <x:c r="A15" s="11" t="s">
-        <x:v>949</x:v>
+        <x:v>947</x:v>
       </x:c>
       <x:c r="B15" s="11" t="s">
-        <x:v>950</x:v>
+        <x:v>948</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="62" hidden="0" customHeight="1">
       <x:c r="A16" s="11" t="s">
-        <x:v>951</x:v>
+        <x:v>949</x:v>
       </x:c>
       <x:c r="B16" s="11" t="s">
-        <x:v>952</x:v>
+        <x:v>950</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="62" hidden="0" customHeight="1">
       <x:c r="A17" s="11" t="s">
-        <x:v>953</x:v>
+        <x:v>951</x:v>
       </x:c>
       <x:c r="B17" s="11" t="s">
-        <x:v>954</x:v>
+        <x:v>952</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="62" hidden="0" customHeight="1">
       <x:c r="A18" s="11" t="s">
-        <x:v>955</x:v>
+        <x:v>953</x:v>
       </x:c>
       <x:c r="B18" s="11" t="s">
-        <x:v>956</x:v>
+        <x:v>954</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="62" hidden="0" customHeight="1">
       <x:c r="A19" s="11" t="s">
-        <x:v>957</x:v>
+        <x:v>955</x:v>
       </x:c>
       <x:c r="B19" s="11" t="s">
-        <x:v>958</x:v>
+        <x:v>956</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" hidden="0" customHeight="1">
       <x:c r="A20" s="11" t="s">
-        <x:v>959</x:v>
+        <x:v>957</x:v>
       </x:c>
       <x:c r="B20" s="11" t="s">
-        <x:v>960</x:v>
+        <x:v>958</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="62" hidden="0" customHeight="1">
       <x:c r="A21" s="11" t="s">
-        <x:v>961</x:v>
+        <x:v>959</x:v>
       </x:c>
       <x:c r="B21" s="11" t="s">
-        <x:v>962</x:v>
+        <x:v>960</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" hidden="0" customHeight="1">
       <x:c r="A22" s="11" t="s">
-        <x:v>963</x:v>
+        <x:v>961</x:v>
       </x:c>
       <x:c r="B22" s="11" t="s">
-        <x:v>964</x:v>
+        <x:v>962</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" hidden="0" customHeight="1">
       <x:c r="A23" s="11" t="s">
-        <x:v>965</x:v>
+        <x:v>963</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
         <x:v>Repository and organisation facts were refreshed through 29 July 2026 for the current GetBible, JoomEngine and Vast Development Method work. The new public state strengthened evidence but introduced no additional independent canonical lineage: 109 unique records and zero fork rows remain authoritative. Final CV production must still recheck time-sensitive present-role, release and conference claims.</x:v>

</xml_diff>